<commit_message>
fix the selection of options in business page drop down
</commit_message>
<xml_diff>
--- a/target/test-classes/TestData.xlsx
+++ b/target/test-classes/TestData.xlsx
@@ -3,12 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2506400\Desktop\Pooja-Workspace\UdemyAutomation\src\test\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{822CED62-4E19-42F4-AC57-46851216540B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{C75C1DEA-AFBD-454E-B052-333317D71C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +13,7 @@
     <sheet name="TestResults" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="C1:N35"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -27,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="210">
   <si>
     <t>extractCategoryCatalog</t>
   </si>
@@ -649,9 +645,6 @@
     <t>Course Publisher</t>
   </si>
   <si>
-    <t>CompanyName</t>
-  </si>
-  <si>
     <t>Cognizant</t>
   </si>
   <si>
@@ -682,27 +675,9 @@
     <t>India</t>
   </si>
   <si>
-    <t>Information Technology</t>
-  </si>
-  <si>
     <t>Free LMS</t>
   </si>
   <si>
-    <t>HR Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Infosys	</t>
-  </si>
-  <si>
-    <t>TCS</t>
-  </si>
-  <si>
-    <t>Learning &amp;Development</t>
-  </si>
-  <si>
-    <t>Banking &amp; Finance</t>
-  </si>
-  <si>
     <t>Singapore</t>
   </si>
   <si>
@@ -728,24 +703,6 @@
   </si>
   <si>
     <t>OrganisationSize</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Government </t>
-  </si>
-  <si>
-    <t>201-500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Private Company </t>
-  </si>
-  <si>
-    <t>51-200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enterprise </t>
-  </si>
-  <si>
-    <t>501-1000</t>
   </si>
   <si>
     <t>API</t>
@@ -793,9 +750,6 @@
     <t>Practical Python Programming for Beginners</t>
   </si>
   <si>
-    <t>This course introduces the fundamentals of Python programming for beginners with no prior coding experience. You will learn how to work with variables, data types, operators, loops, and user input to create simple and functional programs. By the end of the course, you will be able to write complete Python scripts and apply core programming concepts to real-world problems and further learning in software development.</t>
-  </si>
-  <si>
     <t>Expected condition failed: waiting for element to be clickable: By.xpath: //*[contains(text(),'Your Department')] (tried for 20 second(s) with 500 milliseconds interval)
 Build info: version: '4.21.0', revision: '79ed462ef4'
 System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
@@ -831,12 +785,6 @@
     <t>2026-07-22 17:37:06</t>
   </si>
   <si>
-    <t>Python for Data Science: From the Basics to Advanced</t>
-  </si>
-  <si>
-    <t>Python is one of the best and fastest-growing programming languages used in data analysis worldwide. This free online course shows you how to apply the fundamental programming concepts of Python such as looping, variables, data types and data structures to data science. It also explores the NumPy and Pandas libraries that will help you further manipulate, analyze and visualize data in Python.</t>
-  </si>
-  <si>
     <t>Expected condition failed: waiting for element to be clickable: By.xpath: //*[contains(text(),'Your Department')] (tried for 20 second(s) with 500 milliseconds interval)
 Build info: version: '4.21.0', revision: '79ed462ef4'
 System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
@@ -869,15 +817,6 @@
     <t>2026-07-23 09:15:20</t>
   </si>
   <si>
-    <t>Diploma in E-Commerce Web Development</t>
-  </si>
-  <si>
-    <t>This diploma course teaches you how to develop a website to successfully drive e-commerce. We explain how to build an e-commerce website from scratch using HTML, CSS, Javascript, PHP and SQL. We then show you how to develop advanced e-commerce functionalities to display products online, using simple and effective CSS, PHP and SQL code in any development environment. This course can also help small businesses widen their customer base and grow.</t>
-  </si>
-  <si>
-    <t>FAQs</t>
-  </si>
-  <si>
     <t>Expected condition failed: waiting for element to be clickable: By.xpath: //button[contains(.,'Submit')] (tried for 20 second(s) with 500 milliseconds interval)
 Build info: version: '4.21.0', revision: '79ed462ef4'
 System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
@@ -927,13 +866,49 @@
   </si>
   <si>
     <t>Advanced</t>
+  </si>
+  <si>
+    <t>Human Resources (HR)</t>
+  </si>
+  <si>
+    <t>Education &amp; Training</t>
+  </si>
+  <si>
+    <t>Manufacturing &amp; Engineering</t>
+  </si>
+  <si>
+    <t>Zero Gravity</t>
+  </si>
+  <si>
+    <t>NGO</t>
+  </si>
+  <si>
+    <t>Large Enterprise</t>
+  </si>
+  <si>
+    <t>Government</t>
+  </si>
+  <si>
+    <t>BHEL</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 51 - 100 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 201 - 500 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 501 - 1,000 </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -950,12 +925,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color theme="1"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -996,15 +965,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1307,7 +1273,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1316,72 +1282,63 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="22.6328125" customWidth="1"/>
-    <col min="8" max="8" width="14.90625" customWidth="1"/>
-    <col min="9" max="14" width="8.7265625" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="21.36328125" customWidth="1"/>
-    <col min="16" max="16" width="17.81640625" customWidth="1"/>
-    <col min="17" max="17" width="20.6328125" customWidth="1"/>
-    <col min="18" max="18" width="21.81640625" customWidth="1"/>
-    <col min="19" max="20" width="15.7265625" customWidth="1"/>
-    <col min="21" max="21" width="59.6328125" customWidth="1"/>
+    <col min="8" max="8" width="28.26953125" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" customWidth="1"/>
+    <col min="10" max="10" width="24.90625" customWidth="1"/>
+    <col min="11" max="11" width="20.6328125" customWidth="1"/>
+    <col min="12" max="12" width="21.81640625" customWidth="1"/>
+    <col min="13" max="14" width="15.7265625" customWidth="1"/>
+    <col min="15" max="15" width="59.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="B1" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="T1" s="4" t="s">
+      <c r="H1" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="O1" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="U1" s="4" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -1404,32 +1361,31 @@
         <v>113</v>
       </c>
       <c r="H2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I2" t="s">
         <v>139</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="J2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="L2" t="s">
+        <v>203</v>
+      </c>
+      <c r="M2" t="s">
+        <v>208</v>
+      </c>
+      <c r="N2" t="s">
+        <v>141</v>
+      </c>
       <c r="O2" t="s">
-        <v>140</v>
-      </c>
-      <c r="P2" t="s">
-        <v>141</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="R2" t="s">
-        <v>162</v>
-      </c>
-      <c r="S2" t="s">
-        <v>163</v>
-      </c>
-      <c r="T2" t="s">
         <v>142</v>
       </c>
-      <c r="U2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -1437,7 +1393,7 @@
         <v>114</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>110</v>
@@ -1452,32 +1408,31 @@
         <v>117</v>
       </c>
       <c r="H3" t="s">
-        <v>148</v>
-      </c>
-      <c r="I3" s="3"/>
+        <v>198</v>
+      </c>
+      <c r="I3" t="s">
+        <v>145</v>
+      </c>
+      <c r="J3" t="s">
+        <v>199</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="L3" t="s">
+        <v>202</v>
+      </c>
+      <c r="M3" t="s">
+        <v>207</v>
+      </c>
+      <c r="N3" t="s">
+        <v>144</v>
+      </c>
       <c r="O3" t="s">
-        <v>147</v>
-      </c>
-      <c r="P3" t="s">
-        <v>146</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="R3" t="s">
-        <v>164</v>
-      </c>
-      <c r="S3" t="s">
-        <v>165</v>
-      </c>
-      <c r="T3" t="s">
-        <v>145</v>
-      </c>
-      <c r="U3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
@@ -1500,39 +1455,29 @@
         <v>122</v>
       </c>
       <c r="H4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I4" s="3"/>
+        <v>206</v>
+      </c>
+      <c r="I4" t="s">
+        <v>155</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="L4" t="s">
+        <v>204</v>
+      </c>
+      <c r="M4" t="s">
+        <v>209</v>
+      </c>
+      <c r="N4" t="s">
+        <v>146</v>
+      </c>
       <c r="O4" t="s">
-        <v>168</v>
-      </c>
-      <c r="P4" t="s">
-        <v>152</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="R4" t="s">
-        <v>166</v>
-      </c>
-      <c r="S4" t="s">
-        <v>167</v>
-      </c>
-      <c r="T4" t="s">
-        <v>153</v>
-      </c>
-      <c r="U4" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="I6" s="3"/>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="I7" s="3"/>
+        <v>147</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1542,7 +1487,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.08984375" customWidth="1"/>
@@ -1575,121 +1520,6 @@
       </c>
       <c r="G1" s="1" t="s">
         <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>179</v>
-      </c>
-      <c r="C2" t="s">
-        <v>180</v>
-      </c>
-      <c r="D2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E2" t="s">
-        <v>176</v>
-      </c>
-      <c r="F2" t="s">
-        <v>176</v>
-      </c>
-      <c r="G2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>191</v>
-      </c>
-      <c r="C3" t="s">
-        <v>192</v>
-      </c>
-      <c r="D3" t="s">
-        <v>176</v>
-      </c>
-      <c r="E3" t="s">
-        <v>176</v>
-      </c>
-      <c r="F3" t="s">
-        <v>176</v>
-      </c>
-      <c r="G3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>202</v>
-      </c>
-      <c r="C4" t="s">
-        <v>203</v>
-      </c>
-      <c r="D4" t="s">
-        <v>176</v>
-      </c>
-      <c r="E4" t="s">
-        <v>176</v>
-      </c>
-      <c r="F4" t="s">
-        <v>176</v>
-      </c>
-      <c r="G4" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>179</v>
-      </c>
-      <c r="C5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" t="s">
-        <v>176</v>
-      </c>
-      <c r="E5" t="s">
-        <v>176</v>
-      </c>
-      <c r="F5" t="s">
-        <v>176</v>
-      </c>
-      <c r="G5" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>191</v>
-      </c>
-      <c r="C6" t="s">
-        <v>192</v>
-      </c>
-      <c r="D6" t="s">
-        <v>176</v>
-      </c>
-      <c r="E6" t="s">
-        <v>176</v>
-      </c>
-      <c r="F6" t="s">
-        <v>176</v>
-      </c>
-      <c r="G6" t="s">
-        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -2914,7 +2744,7 @@
         <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="D53" t="s">
         <v>3</v>
@@ -2926,7 +2756,7 @@
         <v>4</v>
       </c>
       <c r="G53" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
@@ -2937,7 +2767,7 @@
         <v>1</v>
       </c>
       <c r="C54" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="D54" t="s">
         <v>3</v>
@@ -2949,7 +2779,7 @@
         <v>4</v>
       </c>
       <c r="G54" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
@@ -2960,7 +2790,7 @@
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="D55" t="s">
         <v>3</v>
@@ -2972,7 +2802,7 @@
         <v>4</v>
       </c>
       <c r="G55" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
@@ -2983,7 +2813,7 @@
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="D56" t="s">
         <v>3</v>
@@ -2995,7 +2825,7 @@
         <v>4</v>
       </c>
       <c r="G56" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
@@ -3003,22 +2833,22 @@
         <v>15</v>
       </c>
       <c r="B57" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C57" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="D57" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="E57" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="F57" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G57" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
@@ -3026,22 +2856,22 @@
         <v>15</v>
       </c>
       <c r="B58" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C58" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="D58" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="E58" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="F58" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G58" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
@@ -3052,7 +2882,7 @@
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="D59" t="s">
         <v>3</v>
@@ -3064,7 +2894,7 @@
         <v>4</v>
       </c>
       <c r="G59" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
@@ -3072,22 +2902,22 @@
         <v>18</v>
       </c>
       <c r="B60" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C60" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="D60" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="E60" t="s">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="F60" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G60" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
@@ -3095,22 +2925,22 @@
         <v>18</v>
       </c>
       <c r="B61" t="s">
+        <v>162</v>
+      </c>
+      <c r="C61" t="s">
+        <v>173</v>
+      </c>
+      <c r="D61" t="s">
+        <v>174</v>
+      </c>
+      <c r="E61" t="s">
         <v>175</v>
       </c>
-      <c r="C61" t="s">
-        <v>187</v>
-      </c>
-      <c r="D61" t="s">
-        <v>188</v>
-      </c>
-      <c r="E61" t="s">
-        <v>189</v>
-      </c>
       <c r="F61" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G61" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
@@ -3121,7 +2951,7 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="D62" t="s">
         <v>3</v>
@@ -3133,7 +2963,7 @@
         <v>4</v>
       </c>
       <c r="G62" t="s">
-        <v>194</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
@@ -3141,22 +2971,22 @@
         <v>12</v>
       </c>
       <c r="B63" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C63" t="s">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="D63" t="s">
-        <v>196</v>
+        <v>180</v>
       </c>
       <c r="E63" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="F63" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G63" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
@@ -3164,22 +2994,22 @@
         <v>12</v>
       </c>
       <c r="B64" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C64" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="D64" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="E64" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="F64" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G64" t="s">
-        <v>199</v>
+        <v>183</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
@@ -3187,22 +3017,22 @@
         <v>12</v>
       </c>
       <c r="B65" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C65" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="D65" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="E65" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="F65" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G65" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
@@ -3210,22 +3040,22 @@
         <v>12</v>
       </c>
       <c r="B66" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C66" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="D66" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="E66" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="F66" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G66" t="s">
-        <v>201</v>
+        <v>185</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
@@ -3236,7 +3066,7 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>205</v>
+        <v>186</v>
       </c>
       <c r="D67" t="s">
         <v>3</v>
@@ -3248,7 +3078,7 @@
         <v>4</v>
       </c>
       <c r="G67" t="s">
-        <v>206</v>
+        <v>187</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
@@ -3256,22 +3086,22 @@
         <v>15</v>
       </c>
       <c r="B68" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C68" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="D68" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="E68" t="s">
-        <v>207</v>
+        <v>188</v>
       </c>
       <c r="F68" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G68" t="s">
-        <v>208</v>
+        <v>189</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
@@ -3279,22 +3109,22 @@
         <v>15</v>
       </c>
       <c r="B69" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C69" t="s">
-        <v>209</v>
+        <v>190</v>
       </c>
       <c r="D69" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="E69" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="F69" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G69" t="s">
-        <v>210</v>
+        <v>191</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
@@ -3305,7 +3135,7 @@
         <v>1</v>
       </c>
       <c r="C70" t="s">
-        <v>211</v>
+        <v>192</v>
       </c>
       <c r="D70" t="s">
         <v>3</v>
@@ -3317,7 +3147,7 @@
         <v>4</v>
       </c>
       <c r="G70" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
@@ -3325,22 +3155,22 @@
         <v>18</v>
       </c>
       <c r="B71" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C71" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="D71" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="E71" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="F71" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G71" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
@@ -3348,22 +3178,22 @@
         <v>18</v>
       </c>
       <c r="B72" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="C72" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="D72" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="E72" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="F72" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="G72" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
@@ -3374,7 +3204,7 @@
         <v>1</v>
       </c>
       <c r="C73" t="s">
-        <v>214</v>
+        <v>195</v>
       </c>
       <c r="D73" t="s">
         <v>3</v>
@@ -3386,7 +3216,7 @@
         <v>4</v>
       </c>
       <c r="G73" t="s">
-        <v>215</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update POM structure by using page factory
</commit_message>
<xml_diff>
--- a/target/test-classes/TestData.xlsx
+++ b/target/test-classes/TestData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="326">
   <si>
     <t>extractCategoryCatalog</t>
   </si>
@@ -1192,6 +1192,150 @@
   </si>
   <si>
     <t>2026-07-23 18:44:21</t>
+  </si>
+  <si>
+    <t>stale element reference: stale element not found in the current frame
+  (Session info: chrome=150.0.7871.47)
+For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#stale-element-reference-exception
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Command: [67a854d01c4003a4f5944fd9f86775ed, isElementDisplayed {id=f.5B4CBD3216A188CB8A12625D7E03650C.d.59E7493151B423DFC710FDCB05D907C6.e.1697}]
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.47, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:55535}, goog:processID: 25760, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:55535/devtoo..., se:cdpVersion: 150.0.7871.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Element: [[ChromeDriver: chrome on windows (67a854d01c4003a4f5944fd9f86775ed)] -&gt; xpath: //div[contains(@class,'card--white')]]
+Session ID: 67a854d01c4003a4f5944fd9f86775ed</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:43:32</t>
+  </si>
+  <si>
+    <t>stale element reference: stale element not found in the current frame
+  (Session info: chrome=150.0.7871.47)
+For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#stale-element-reference-exception
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Command: [ecd22cd6a781d5c71bdf92d1acba74cd, isElementDisplayed {id=f.BDCA8E81CF035C786D0E40226717BBB9.d.CA4255D9BDD09D2BB86CEC09E6B6F3B5.e.1713}]
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.47, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:53529}, goog:processID: 29588, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:53529/devtoo..., se:cdpVersion: 150.0.7871.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Element: [[ChromeDriver: chrome on windows (ecd22cd6a781d5c71bdf92d1acba74cd)] -&gt; xpath: //div[contains(@class,'card--white')]]
+Session ID: ecd22cd6a781d5c71bdf92d1acba74cd</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:44:13</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:44:52</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:45:35</t>
+  </si>
+  <si>
+    <t>2026-07-23 19:46:15</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for element to be clickable: By.xpath: //div[@data-url-var='level']//label[contains(translate(normalize-space(.),'ABCDEFGHIJKLMNOPQRSTUVWXYZ','abcdefghijklmnopqrstuvwxyz'),'beginner')] (tried for 20 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.47, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:65441}, goog:processID: 22588, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:65441/devtoo..., se:cdpVersion: 150.0.7871.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 9f3e34de88f1a82cbfef74e2fd2f98d4</t>
+  </si>
+  <si>
+    <t>2026-07-24 09:08:51</t>
+  </si>
+  <si>
+    <t>2026-07-24 09:09:20</t>
+  </si>
+  <si>
+    <t>2026-07-24 09:09:21</t>
+  </si>
+  <si>
+    <t>2026-07-24 09:10:02</t>
+  </si>
+  <si>
+    <t>2026-07-24 09:10:37</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for element to be clickable: By.xpath: //div[@data-url-var='level']//label[contains(translate(normalize-space(.),'ABCDEFGHIJKLMNOPQRSTUVWXYZ','abcdefghijklmnopqrstuvwxyz'),'intermediate')] (tried for 20 second(s) with 500 milliseconds interval)
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.47, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50202}, goog:processID: 17984, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:50202/devtoo..., se:cdpVersion: 150.0.7871.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: f5bd8b62212cf18adba3ead9f99b660b</t>
+  </si>
+  <si>
+    <t>2026-07-24 09:11:27</t>
+  </si>
+  <si>
+    <t>2026-07-24 10:30:19</t>
+  </si>
+  <si>
+    <t>2026-07-24 10:30:20</t>
+  </si>
+  <si>
+    <t>Unable to enter value : Aisha</t>
+  </si>
+  <si>
+    <t>2026-07-24 10:30:40</t>
+  </si>
+  <si>
+    <t>2026-07-24 10:31:09</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Unable to enter value : Rohan</t>
+  </si>
+  <si>
+    <t>2026-07-24 10:32:02</t>
+  </si>
+  <si>
+    <t>no such element: Unable to locate element: {"method":"xpath","selector":"//div[@data-url-var='translation']"}
+  (Session info: chrome=150.0.7871.47)
+For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#no-such-element-exception
+Build info: version: '4.21.0', revision: '79ed462ef4'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.10'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Command: [37a2434c184bf4829ca6ea27d2fb4f98, findElement {value=//div[@data-url-var='translation'], using=xpath}]
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.47, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\2506400\AppData\Lo...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:51412}, goog:processID: 27588, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:51412/devtoo..., se:cdpVersion: 150.0.7871.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 37a2434c184bf4829ca6ea27d2fb4f98</t>
+  </si>
+  <si>
+    <t>2026-07-24 10:32:28</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:03:52</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:03:54</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:04:15</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:04:29</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:04:58</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:04:59</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:05:22</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:05:38</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:06:07</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:06:30</t>
+  </si>
+  <si>
+    <t>2026-07-24 11:06:48</t>
   </si>
 </sst>
 </file>
@@ -1807,7 +1951,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BFA3FA-6A41-46D8-9F46-57C4912E9286}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="14.08984375"/>
@@ -2095,6 +2239,167 @@
         <v>235</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>234</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="G14" t="s" s="0">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>214</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="F15" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="G15" t="s" s="0">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="F16" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="G16" t="s" s="0">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>214</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="F17" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="G17" t="s" s="0">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="F18" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="G18" t="s" s="0">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="F19" t="s" s="0">
+        <v>234</v>
+      </c>
+      <c r="G19" t="s" s="0">
+        <v>235</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2102,7 +2407,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G125"/>
+  <dimension ref="A1:G161"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" customWidth="true" width="12.0"/>
@@ -4988,6 +5293,834 @@
         <v>289</v>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B126" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C126" t="s" s="0">
+        <v>290</v>
+      </c>
+      <c r="D126" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E126" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F126" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G126" t="s" s="0">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B127" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C127" t="s" s="0">
+        <v>292</v>
+      </c>
+      <c r="D127" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E127" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F127" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G127" t="s" s="0">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B128" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C128" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="D128" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E128" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="F128" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G128" t="s" s="0">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B129" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C129" t="s" s="0">
+        <v>171</v>
+      </c>
+      <c r="D129" t="s" s="0">
+        <v>172</v>
+      </c>
+      <c r="E129" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="F129" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G129" t="s" s="0">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B130" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C130" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D130" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E130" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F130" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G130" t="s" s="0">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B131" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="C131" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D131" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E131" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F131" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G131" t="s" s="0">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B132" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C132" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D132" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E132" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F132" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G132" t="s" s="0">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B133" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C133" t="s" s="0">
+        <v>297</v>
+      </c>
+      <c r="D133" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E133" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F133" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G133" t="s" s="0">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B134" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C134" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D134" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E134" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F134" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G134" t="s" s="0">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B135" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C135" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="D135" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="E135" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F135" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G135" t="s" s="0">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B136" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C136" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D136" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E136" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F136" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G136" t="s" s="0">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B137" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="C137" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D137" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E137" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F137" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G137" t="s" s="0">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B138" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C138" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D138" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E138" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F138" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G138" t="s" s="0">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B139" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C139" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D139" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E139" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F139" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G139" t="s" s="0">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B140" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C140" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="D140" t="s" s="0">
+        <v>178</v>
+      </c>
+      <c r="E140" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="F140" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G140" t="s" s="0">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B141" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C141" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="D141" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="E141" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="F141" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G141" t="s" s="0">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B142" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C142" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="D142" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E142" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F142" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G142" t="s" s="0">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B143" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C143" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="D143" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E143" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="F143" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G143" t="s" s="0">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B144" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C144" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="D144" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="E144" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="F144" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G144" t="s" s="0">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B145" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C145" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="D145" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E145" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F145" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G145" t="s" s="0">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B146" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C146" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D146" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E146" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F146" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G146" t="s" s="0">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B147" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C147" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="D147" t="s" s="0">
+        <v>178</v>
+      </c>
+      <c r="E147" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="F147" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G147" t="s" s="0">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B148" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C148" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="D148" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="E148" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="F148" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G148" t="s" s="0">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B149" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C149" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D149" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E149" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F149" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G149" t="s" s="0">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B150" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="C150" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D150" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E150" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F150" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G150" t="s" s="0">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B151" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C151" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D151" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E151" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F151" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G151" t="s" s="0">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B152" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C152" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="D152" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E152" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="F152" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G152" t="s" s="0">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B153" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C153" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="D153" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="E153" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="F153" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G153" t="s" s="0">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B154" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C154" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D154" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E154" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F154" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G154" t="s" s="0">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B155" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="C155" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D155" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E155" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F155" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G155" t="s" s="0">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B156" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C156" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D156" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E156" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F156" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G156" t="s" s="0">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B157" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C157" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="D157" t="s" s="0">
+        <v>168</v>
+      </c>
+      <c r="E157" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="F157" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G157" t="s" s="0">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B158" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="C158" t="s" s="0">
+        <v>171</v>
+      </c>
+      <c r="D158" t="s" s="0">
+        <v>172</v>
+      </c>
+      <c r="E158" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="F158" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G158" t="s" s="0">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B159" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="C159" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D159" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E159" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F159" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="G159" t="s" s="0">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B160" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="C160" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D160" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E160" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F160" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G160" t="s" s="0">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B161" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C161" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="D161" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E161" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="F161" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="G161" t="s" s="0">
+        <v>325</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>